<commit_message>
Propuesta: curva completa sin ceros, −5% cantidades, rango KIDS alineado
- Todas las tallas rellenadas por curva (Tucupido CAB/KIDS incluido)
- Ajuste proporcional −5% sobre totales calculados
- MÁXIMO ×1.2 igual en CAB y KIDS (~20% rango en ambos)
- Evita recorte que aplanaba curvas KIDS al mínimo 4

Co-authored-by: scm-svg <scm-svg@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/PROPUESTA_PRODUCCION_SUBLIMADO_ACTUALIZADA.xlsx
+++ b/PROPUESTA_PRODUCCION_SUBLIMADO_ACTUALIZADA.xlsx
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -496,6 +496,11 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
+          <t>% Rango</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
           <t>Δ vs equipo</t>
         </is>
       </c>
@@ -510,16 +515,19 @@
         <v>349</v>
       </c>
       <c r="C2" t="n">
-        <v>524</v>
+        <v>474</v>
       </c>
       <c r="D2" t="n">
-        <v>637</v>
+        <v>568</v>
       </c>
       <c r="E2" t="n">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="F2" t="n">
-        <v>175</v>
+        <v>19.8</v>
+      </c>
+      <c r="G2" t="n">
+        <v>125</v>
       </c>
     </row>
     <row r="3">
@@ -532,16 +540,19 @@
         <v>136</v>
       </c>
       <c r="C3" t="n">
-        <v>248</v>
+        <v>225</v>
       </c>
       <c r="D3" t="n">
-        <v>307</v>
+        <v>274</v>
       </c>
       <c r="E3" t="n">
-        <v>59</v>
+        <v>49</v>
       </c>
       <c r="F3" t="n">
-        <v>112</v>
+        <v>21.8</v>
+      </c>
+      <c r="G3" t="n">
+        <v>89</v>
       </c>
     </row>
     <row r="4">
@@ -554,16 +565,19 @@
         <v>485</v>
       </c>
       <c r="C4" t="n">
-        <v>772</v>
+        <v>699</v>
       </c>
       <c r="D4" t="n">
-        <v>944</v>
+        <v>842</v>
       </c>
       <c r="E4" t="n">
-        <v>172</v>
+        <v>143</v>
       </c>
       <c r="F4" t="n">
-        <v>287</v>
+        <v>20.5</v>
+      </c>
+      <c r="G4" t="n">
+        <v>214</v>
       </c>
     </row>
   </sheetData>
@@ -650,19 +664,19 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="C6" s="5" t="n">
+        <v>31</v>
+      </c>
+      <c r="D6" s="5" t="n">
         <v>38</v>
       </c>
-      <c r="D6" s="5" t="n">
-        <v>37</v>
-      </c>
       <c r="E6" s="5" t="n">
+        <v>19</v>
+      </c>
+      <c r="F6" s="5" t="n">
         <v>13</v>
-      </c>
-      <c r="F6" s="5" t="n">
-        <v>14</v>
       </c>
       <c r="G6" s="6">
         <f>SUM(B6:F6)</f>
@@ -707,19 +721,19 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C8" s="5" t="n">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="D8" s="5" t="n">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="F8" s="5" t="n">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="G8" s="6">
         <f>SUM(B8:F8)</f>
@@ -763,14 +777,20 @@
           <t>Tucupido — MÍNIMO</t>
         </is>
       </c>
+      <c r="B10" s="5" t="n">
+        <v>4</v>
+      </c>
       <c r="C10" s="5" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="D10" s="5" t="n">
-        <v>20</v>
+        <v>14</v>
+      </c>
+      <c r="E10" s="5" t="n">
+        <v>7</v>
       </c>
       <c r="F10" s="5" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G10" s="6">
         <f>SUM(B10:F10)</f>
@@ -815,19 +835,19 @@
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>26</v>
+        <v>12</v>
       </c>
       <c r="C12" s="5" t="n">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="D12" s="5" t="n">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="G12" s="6">
         <f>SUM(B12:F12)</f>
@@ -1035,13 +1055,13 @@
         <v>4</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="G6" s="5" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I6" s="6">
         <f>SUM(B6:H6)</f>
@@ -1109,10 +1129,10 @@
         <v>4</v>
       </c>
       <c r="G8" s="5" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="I8" s="6">
         <f>SUM(B8:H8)</f>
@@ -1164,11 +1184,26 @@
           <t>Tucupido — MÍNIMO</t>
         </is>
       </c>
+      <c r="B10" s="5" t="n">
+        <v>4</v>
+      </c>
       <c r="C10" s="5" t="n">
-        <v>11</v>
+        <v>4</v>
+      </c>
+      <c r="D10" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="E10" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="F10" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="G10" s="5" t="n">
+        <v>4</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I10" s="6">
         <f>SUM(B10:H10)</f>
@@ -1221,25 +1256,25 @@
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="C12" s="5" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D12" s="5" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="G12" s="5" t="n">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="I12" s="6">
         <f>SUM(B12:H12)</f>
@@ -1374,7 +1409,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1419,10 +1454,10 @@
         <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="E2" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3">
@@ -1440,10 +1475,10 @@
         <v>24</v>
       </c>
       <c r="D3" t="n">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="E3" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4">
@@ -1461,10 +1496,10 @@
         <v>28</v>
       </c>
       <c r="D4" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="E4" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5">
@@ -1482,10 +1517,10 @@
         <v>10</v>
       </c>
       <c r="D5" t="n">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="E5" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6">
@@ -1503,10 +1538,10 @@
         <v>10</v>
       </c>
       <c r="D6" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7">
@@ -1524,10 +1559,10 @@
         <v>0</v>
       </c>
       <c r="D7" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="E7" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="8">
@@ -1545,10 +1580,10 @@
         <v>15</v>
       </c>
       <c r="D8" t="n">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="E8" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="9">
@@ -1566,10 +1601,10 @@
         <v>30</v>
       </c>
       <c r="D9" t="n">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="E9" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="10">
@@ -1587,10 +1622,10 @@
         <v>21</v>
       </c>
       <c r="D10" t="n">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="E10" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -1608,10 +1643,10 @@
         <v>16</v>
       </c>
       <c r="D11" t="n">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="E11" t="n">
-        <v>5</v>
+        <v>-3</v>
       </c>
     </row>
     <row r="12">
@@ -1622,17 +1657,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="D12" t="n">
-        <v>20</v>
+        <v>4</v>
       </c>
       <c r="E12" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="13">
@@ -1643,17 +1678,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>M</t>
         </is>
       </c>
       <c r="C13" t="n">
         <v>15</v>
       </c>
       <c r="D13" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="E13" t="n">
-        <v>5</v>
+        <v>-3</v>
       </c>
     </row>
     <row r="14">
@@ -1664,59 +1699,59 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2XL</t>
+          <t>L</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="D14" t="n">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="E14" t="n">
-        <v>4</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Nuevo color</t>
+          <t>Tucupido</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>XL</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="D15" t="n">
-        <v>26</v>
+        <v>7</v>
       </c>
       <c r="E15" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Nuevo color</t>
+          <t>Tucupido</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>2XL</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>45</v>
+        <v>0</v>
       </c>
       <c r="D16" t="n">
-        <v>64</v>
+        <v>6</v>
       </c>
       <c r="E16" t="n">
-        <v>19</v>
+        <v>6</v>
       </c>
     </row>
     <row r="17">
@@ -1727,17 +1762,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>S</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>45</v>
+        <v>20</v>
       </c>
       <c r="D17" t="n">
-        <v>77</v>
+        <v>12</v>
       </c>
       <c r="E17" t="n">
-        <v>32</v>
+        <v>-8</v>
       </c>
     </row>
     <row r="18">
@@ -1748,17 +1783,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>XL</t>
+          <t>M</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="D18" t="n">
-        <v>46</v>
+        <v>61</v>
       </c>
       <c r="E18" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
     </row>
     <row r="19">
@@ -1769,17 +1804,59 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>45</v>
+      </c>
+      <c r="D19" t="n">
+        <v>73</v>
+      </c>
+      <c r="E19" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Nuevo color</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>XL</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>35</v>
+      </c>
+      <c r="D20" t="n">
+        <v>36</v>
+      </c>
+      <c r="E20" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Nuevo color</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
           <t>2XL</t>
         </is>
       </c>
-      <c r="C19" t="n">
+      <c r="C21" t="n">
         <v>20</v>
       </c>
-      <c r="D19" t="n">
-        <v>26</v>
-      </c>
-      <c r="E19" t="n">
-        <v>6</v>
+      <c r="D21" t="n">
+        <v>24</v>
+      </c>
+      <c r="E21" t="n">
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -1793,7 +1870,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1922,10 +1999,10 @@
         <v>8</v>
       </c>
       <c r="D6" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="E6" t="n">
-        <v>3</v>
+        <v>-4</v>
       </c>
     </row>
     <row r="7">
@@ -1943,10 +2020,10 @@
         <v>0</v>
       </c>
       <c r="D7" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="E7" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8">
@@ -1964,10 +2041,10 @@
         <v>0</v>
       </c>
       <c r="D8" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E8" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9">
@@ -2090,10 +2167,10 @@
         <v>0</v>
       </c>
       <c r="D14" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="E14" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="15">
@@ -2111,10 +2188,10 @@
         <v>8</v>
       </c>
       <c r="D15" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="E15" t="n">
-        <v>3</v>
+        <v>-2</v>
       </c>
     </row>
     <row r="16">
@@ -2125,17 +2202,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="D16" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="E16" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="17">
@@ -2146,122 +2223,122 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="D17" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E17" t="n">
-        <v>1</v>
+        <v>-4</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Nuevo color</t>
+          <t>Tucupido</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>6</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="D18" t="n">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="E18" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Nuevo color</t>
+          <t>Tucupido</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>8</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="D19" t="n">
-        <v>20</v>
+        <v>4</v>
       </c>
       <c r="E19" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Nuevo color</t>
+          <t>Tucupido</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>10</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="D20" t="n">
-        <v>21</v>
+        <v>4</v>
       </c>
       <c r="E20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Nuevo color</t>
+          <t>Tucupido</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>12</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="D21" t="n">
-        <v>21</v>
+        <v>4</v>
       </c>
       <c r="E21" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Nuevo color</t>
+          <t>Tucupido</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>14</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="D22" t="n">
-        <v>21</v>
+        <v>6</v>
       </c>
       <c r="E22" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="23">
@@ -2272,17 +2349,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="D23" t="n">
-        <v>26</v>
+        <v>10</v>
       </c>
       <c r="E23" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24">
@@ -2293,17 +2370,122 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>10</v>
+      </c>
+      <c r="D24" t="n">
+        <v>19</v>
+      </c>
+      <c r="E24" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Nuevo color</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>16</v>
+      </c>
+      <c r="D25" t="n">
+        <v>19</v>
+      </c>
+      <c r="E25" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Nuevo color</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>16</v>
+      </c>
+      <c r="D26" t="n">
+        <v>19</v>
+      </c>
+      <c r="E26" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Nuevo color</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>16</v>
+      </c>
+      <c r="D27" t="n">
+        <v>19</v>
+      </c>
+      <c r="E27" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Nuevo color</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>20</v>
+      </c>
+      <c r="D28" t="n">
+        <v>19</v>
+      </c>
+      <c r="E28" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Nuevo color</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
           <t>14</t>
         </is>
       </c>
-      <c r="C24" t="n">
+      <c r="C29" t="n">
         <v>20</v>
       </c>
-      <c r="D24" t="n">
-        <v>32</v>
-      </c>
-      <c r="E24" t="n">
-        <v>12</v>
+      <c r="D29" t="n">
+        <v>30</v>
+      </c>
+      <c r="E29" t="n">
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Distribuir propuesta por mix de ventas del dashboard (tallas KIDS)
- Pesos por talla desde ventas Mar–Ago 2026 (meses velocidad del dashboard)
- Nuevo color usa pool Playuela+Sal+Tucupido+Sombrero
- Total mínimo calculado para respetar piso 4 sin aplanar curvas
- KIDS deja de tener cantidades idénticas; CAB/Tucupido XL alineado a ventas

Co-authored-by: scm-svg <scm-svg@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/PROPUESTA_PRODUCCION_SUBLIMADO_ACTUALIZADA.xlsx
+++ b/PROPUESTA_PRODUCCION_SUBLIMADO_ACTUALIZADA.xlsx
@@ -515,19 +515,19 @@
         <v>349</v>
       </c>
       <c r="C2" t="n">
-        <v>474</v>
+        <v>472</v>
       </c>
       <c r="D2" t="n">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="E2" t="n">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="F2" t="n">
-        <v>19.8</v>
+        <v>20.1</v>
       </c>
       <c r="G2" t="n">
-        <v>125</v>
+        <v>123</v>
       </c>
     </row>
     <row r="3">
@@ -540,19 +540,19 @@
         <v>136</v>
       </c>
       <c r="C3" t="n">
-        <v>225</v>
+        <v>305</v>
       </c>
       <c r="D3" t="n">
-        <v>274</v>
+        <v>366</v>
       </c>
       <c r="E3" t="n">
-        <v>49</v>
+        <v>61</v>
       </c>
       <c r="F3" t="n">
-        <v>21.8</v>
+        <v>20</v>
       </c>
       <c r="G3" t="n">
-        <v>89</v>
+        <v>169</v>
       </c>
     </row>
     <row r="4">
@@ -565,19 +565,19 @@
         <v>485</v>
       </c>
       <c r="C4" t="n">
-        <v>699</v>
+        <v>777</v>
       </c>
       <c r="D4" t="n">
-        <v>842</v>
+        <v>933</v>
       </c>
       <c r="E4" t="n">
-        <v>143</v>
+        <v>156</v>
       </c>
       <c r="F4" t="n">
-        <v>20.5</v>
+        <v>20.1</v>
       </c>
       <c r="G4" t="n">
-        <v>214</v>
+        <v>292</v>
       </c>
     </row>
   </sheetData>
@@ -664,13 +664,13 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="C6" s="5" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D6" s="5" t="n">
-        <v>38</v>
+        <v>28</v>
       </c>
       <c r="E6" s="5" t="n">
         <v>19</v>
@@ -721,19 +721,19 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="C8" s="5" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D8" s="5" t="n">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="F8" s="5" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G8" s="6">
         <f>SUM(B8:F8)</f>
@@ -778,19 +778,19 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="C10" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="D10" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="E10" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="F10" s="5" t="n">
         <v>4</v>
-      </c>
-      <c r="C10" s="5" t="n">
-        <v>12</v>
-      </c>
-      <c r="D10" s="5" t="n">
-        <v>14</v>
-      </c>
-      <c r="E10" s="5" t="n">
-        <v>7</v>
-      </c>
-      <c r="F10" s="5" t="n">
-        <v>6</v>
       </c>
       <c r="G10" s="6">
         <f>SUM(B10:F10)</f>
@@ -835,19 +835,19 @@
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>12</v>
+        <v>28</v>
       </c>
       <c r="C12" s="5" t="n">
         <v>61</v>
       </c>
       <c r="D12" s="5" t="n">
-        <v>73</v>
+        <v>60</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G12" s="6">
         <f>SUM(B12:F12)</f>
@@ -1043,22 +1043,22 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C6" s="5" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D6" s="5" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="E6" s="5" t="n">
         <v>4</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G6" s="5" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="H6" s="5" t="n">
         <v>6</v>
@@ -1114,25 +1114,25 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C8" s="5" t="n">
         <v>4</v>
       </c>
       <c r="D8" s="5" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="F8" s="5" t="n">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="G8" s="5" t="n">
-        <v>4</v>
+        <v>21</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="I8" s="6">
         <f>SUM(B8:H8)</f>
@@ -1194,10 +1194,10 @@
         <v>4</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F10" s="5" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G10" s="5" t="n">
         <v>4</v>
@@ -1256,25 +1256,25 @@
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="C12" s="5" t="n">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="D12" s="5" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="G12" s="5" t="n">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="I12" s="6">
         <f>SUM(B12:H12)</f>
@@ -1454,10 +1454,10 @@
         <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="E2" t="n">
-        <v>6</v>
+        <v>15</v>
       </c>
     </row>
     <row r="3">
@@ -1475,10 +1475,10 @@
         <v>24</v>
       </c>
       <c r="D3" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E3" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="4">
@@ -1496,10 +1496,10 @@
         <v>28</v>
       </c>
       <c r="D4" t="n">
-        <v>38</v>
+        <v>28</v>
       </c>
       <c r="E4" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -1559,10 +1559,10 @@
         <v>0</v>
       </c>
       <c r="D7" t="n">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="E7" t="n">
-        <v>7</v>
+        <v>17</v>
       </c>
     </row>
     <row r="8">
@@ -1580,10 +1580,10 @@
         <v>15</v>
       </c>
       <c r="D8" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E8" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="9">
@@ -1601,10 +1601,10 @@
         <v>30</v>
       </c>
       <c r="D9" t="n">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="E9" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
     </row>
     <row r="10">
@@ -1622,10 +1622,10 @@
         <v>21</v>
       </c>
       <c r="D10" t="n">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="E10" t="n">
-        <v>0</v>
+        <v>-7</v>
       </c>
     </row>
     <row r="11">
@@ -1643,10 +1643,10 @@
         <v>16</v>
       </c>
       <c r="D11" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E11" t="n">
-        <v>-3</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="12">
@@ -1664,10 +1664,10 @@
         <v>0</v>
       </c>
       <c r="D12" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E12" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="13">
@@ -1685,10 +1685,10 @@
         <v>15</v>
       </c>
       <c r="D13" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E13" t="n">
-        <v>-3</v>
+        <v>-5</v>
       </c>
     </row>
     <row r="14">
@@ -1706,10 +1706,10 @@
         <v>15</v>
       </c>
       <c r="D14" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="E14" t="n">
-        <v>-1</v>
+        <v>-5</v>
       </c>
     </row>
     <row r="15">
@@ -1727,10 +1727,10 @@
         <v>0</v>
       </c>
       <c r="D15" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="E15" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
     </row>
     <row r="16">
@@ -1748,10 +1748,10 @@
         <v>0</v>
       </c>
       <c r="D16" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E16" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="17">
@@ -1769,10 +1769,10 @@
         <v>20</v>
       </c>
       <c r="D17" t="n">
-        <v>12</v>
+        <v>28</v>
       </c>
       <c r="E17" t="n">
-        <v>-8</v>
+        <v>8</v>
       </c>
     </row>
     <row r="18">
@@ -1811,10 +1811,10 @@
         <v>45</v>
       </c>
       <c r="D19" t="n">
-        <v>73</v>
+        <v>60</v>
       </c>
       <c r="E19" t="n">
-        <v>28</v>
+        <v>15</v>
       </c>
     </row>
     <row r="20">
@@ -1832,10 +1832,10 @@
         <v>35</v>
       </c>
       <c r="D20" t="n">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="E20" t="n">
-        <v>1</v>
+        <v>-3</v>
       </c>
     </row>
     <row r="21">
@@ -1853,10 +1853,10 @@
         <v>20</v>
       </c>
       <c r="D21" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E21" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -1915,10 +1915,10 @@
         <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3">
@@ -1936,10 +1936,10 @@
         <v>0</v>
       </c>
       <c r="D3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4">
@@ -1957,10 +1957,10 @@
         <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="E4" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5">
@@ -1999,10 +1999,10 @@
         <v>8</v>
       </c>
       <c r="D6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E6" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
     </row>
     <row r="7">
@@ -2020,10 +2020,10 @@
         <v>0</v>
       </c>
       <c r="D7" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="E7" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
     </row>
     <row r="8">
@@ -2062,10 +2062,10 @@
         <v>0</v>
       </c>
       <c r="D9" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="E9" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="10">
@@ -2104,10 +2104,10 @@
         <v>0</v>
       </c>
       <c r="D11" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="E11" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
     </row>
     <row r="12">
@@ -2125,10 +2125,10 @@
         <v>0</v>
       </c>
       <c r="D12" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="E12" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
     </row>
     <row r="13">
@@ -2146,10 +2146,10 @@
         <v>0</v>
       </c>
       <c r="D13" t="n">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="E13" t="n">
-        <v>4</v>
+        <v>19</v>
       </c>
     </row>
     <row r="14">
@@ -2167,10 +2167,10 @@
         <v>0</v>
       </c>
       <c r="D14" t="n">
-        <v>4</v>
+        <v>21</v>
       </c>
       <c r="E14" t="n">
-        <v>4</v>
+        <v>21</v>
       </c>
     </row>
     <row r="15">
@@ -2188,10 +2188,10 @@
         <v>8</v>
       </c>
       <c r="D15" t="n">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="E15" t="n">
-        <v>-2</v>
+        <v>12</v>
       </c>
     </row>
     <row r="16">
@@ -2272,10 +2272,10 @@
         <v>0</v>
       </c>
       <c r="D19" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E19" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="20">
@@ -2293,10 +2293,10 @@
         <v>0</v>
       </c>
       <c r="D20" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E20" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="21">
@@ -2356,10 +2356,10 @@
         <v>10</v>
       </c>
       <c r="D23" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E23" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="24">
@@ -2377,10 +2377,10 @@
         <v>10</v>
       </c>
       <c r="D24" t="n">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="E24" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
     </row>
     <row r="25">
@@ -2398,10 +2398,10 @@
         <v>16</v>
       </c>
       <c r="D25" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="26">
@@ -2419,10 +2419,10 @@
         <v>16</v>
       </c>
       <c r="D26" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E26" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="27">
@@ -2440,10 +2440,10 @@
         <v>16</v>
       </c>
       <c r="D27" t="n">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="E27" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
     </row>
     <row r="28">
@@ -2461,10 +2461,10 @@
         <v>20</v>
       </c>
       <c r="D28" t="n">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="E28" t="n">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="29">
@@ -2482,10 +2482,10 @@
         <v>20</v>
       </c>
       <c r="D29" t="n">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="E29" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Ajustar KIDS −7% proporcional y bajar talla S en CAB (Playuela/Sal/Nuevo)
- KIDS: factor adicional ×0.93 sobre total (mantiene mix de ventas)
- CAB S: ×0.72 en Playuela, Sal y Nuevo color (Tucupido sin cambio)

Co-authored-by: scm-svg <scm-svg@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/PROPUESTA_PRODUCCION_SUBLIMADO_ACTUALIZADA.xlsx
+++ b/PROPUESTA_PRODUCCION_SUBLIMADO_ACTUALIZADA.xlsx
@@ -515,19 +515,19 @@
         <v>349</v>
       </c>
       <c r="C2" t="n">
-        <v>472</v>
+        <v>455</v>
       </c>
       <c r="D2" t="n">
-        <v>567</v>
+        <v>546</v>
       </c>
       <c r="E2" t="n">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="F2" t="n">
-        <v>20.1</v>
+        <v>20</v>
       </c>
       <c r="G2" t="n">
-        <v>123</v>
+        <v>106</v>
       </c>
     </row>
     <row r="3">
@@ -540,19 +540,19 @@
         <v>136</v>
       </c>
       <c r="C3" t="n">
-        <v>305</v>
+        <v>295</v>
       </c>
       <c r="D3" t="n">
-        <v>366</v>
+        <v>354</v>
       </c>
       <c r="E3" t="n">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="F3" t="n">
         <v>20</v>
       </c>
       <c r="G3" t="n">
-        <v>169</v>
+        <v>159</v>
       </c>
     </row>
     <row r="4">
@@ -565,19 +565,19 @@
         <v>485</v>
       </c>
       <c r="C4" t="n">
-        <v>777</v>
+        <v>750</v>
       </c>
       <c r="D4" t="n">
-        <v>933</v>
+        <v>900</v>
       </c>
       <c r="E4" t="n">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="F4" t="n">
-        <v>20.1</v>
+        <v>20</v>
       </c>
       <c r="G4" t="n">
-        <v>292</v>
+        <v>265</v>
       </c>
     </row>
   </sheetData>
@@ -664,7 +664,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="C6" s="5" t="n">
         <v>32</v>
@@ -721,7 +721,7 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="C8" s="5" t="n">
         <v>34</v>
@@ -835,7 +835,7 @@
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="C12" s="5" t="n">
         <v>61</v>
@@ -1256,25 +1256,25 @@
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C12" s="5" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D12" s="5" t="n">
+        <v>19</v>
+      </c>
+      <c r="E12" s="5" t="n">
+        <v>16</v>
+      </c>
+      <c r="F12" s="5" t="n">
+        <v>21</v>
+      </c>
+      <c r="G12" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="H12" s="5" t="n">
         <v>20</v>
-      </c>
-      <c r="E12" s="5" t="n">
-        <v>18</v>
-      </c>
-      <c r="F12" s="5" t="n">
-        <v>23</v>
-      </c>
-      <c r="G12" s="5" t="n">
-        <v>27</v>
-      </c>
-      <c r="H12" s="5" t="n">
-        <v>21</v>
       </c>
       <c r="I12" s="6">
         <f>SUM(B12:H12)</f>
@@ -1454,10 +1454,10 @@
         <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="E2" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
     </row>
     <row r="3">
@@ -1559,10 +1559,10 @@
         <v>0</v>
       </c>
       <c r="D7" t="n">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="E7" t="n">
-        <v>17</v>
+        <v>12</v>
       </c>
     </row>
     <row r="8">
@@ -1769,10 +1769,10 @@
         <v>20</v>
       </c>
       <c r="D17" t="n">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="E17" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
@@ -2356,10 +2356,10 @@
         <v>10</v>
       </c>
       <c r="D23" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E23" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="24">
@@ -2377,10 +2377,10 @@
         <v>10</v>
       </c>
       <c r="D24" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E24" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25">
@@ -2398,10 +2398,10 @@
         <v>16</v>
       </c>
       <c r="D25" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="26">
@@ -2419,10 +2419,10 @@
         <v>16</v>
       </c>
       <c r="D26" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E26" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27">
@@ -2440,10 +2440,10 @@
         <v>16</v>
       </c>
       <c r="D27" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="E27" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="28">
@@ -2461,10 +2461,10 @@
         <v>20</v>
       </c>
       <c r="D28" t="n">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E28" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="29">
@@ -2482,10 +2482,10 @@
         <v>20</v>
       </c>
       <c r="D29" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E29" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
KIDS: recorte adicional −8% por talla (×0.92 sobre cantidades finales)
Aplica el trim directamente en cada talla para que baje aunque
el color esté en el piso mínimo proporcional.

Co-authored-by: scm-svg <scm-svg@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/PROPUESTA_PRODUCCION_SUBLIMADO_ACTUALIZADA.xlsx
+++ b/PROPUESTA_PRODUCCION_SUBLIMADO_ACTUALIZADA.xlsx
@@ -540,19 +540,19 @@
         <v>136</v>
       </c>
       <c r="C3" t="n">
-        <v>295</v>
+        <v>273</v>
       </c>
       <c r="D3" t="n">
-        <v>354</v>
+        <v>330</v>
       </c>
       <c r="E3" t="n">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="F3" t="n">
-        <v>20</v>
+        <v>20.9</v>
       </c>
       <c r="G3" t="n">
-        <v>159</v>
+        <v>137</v>
       </c>
     </row>
     <row r="4">
@@ -565,19 +565,19 @@
         <v>485</v>
       </c>
       <c r="C4" t="n">
-        <v>750</v>
+        <v>728</v>
       </c>
       <c r="D4" t="n">
-        <v>900</v>
+        <v>876</v>
       </c>
       <c r="E4" t="n">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="F4" t="n">
-        <v>20</v>
+        <v>20.3</v>
       </c>
       <c r="G4" t="n">
-        <v>265</v>
+        <v>243</v>
       </c>
     </row>
   </sheetData>
@@ -1049,7 +1049,7 @@
         <v>5</v>
       </c>
       <c r="D6" s="5" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E6" s="5" t="n">
         <v>4</v>
@@ -1058,7 +1058,7 @@
         <v>5</v>
       </c>
       <c r="G6" s="5" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="H6" s="5" t="n">
         <v>6</v>
@@ -1114,25 +1114,25 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C8" s="5" t="n">
         <v>4</v>
       </c>
       <c r="D8" s="5" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F8" s="5" t="n">
+        <v>17</v>
+      </c>
+      <c r="G8" s="5" t="n">
         <v>19</v>
       </c>
-      <c r="G8" s="5" t="n">
-        <v>21</v>
-      </c>
       <c r="H8" s="5" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="I8" s="6">
         <f>SUM(B8:H8)</f>
@@ -1256,25 +1256,25 @@
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C12" s="5" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D12" s="5" t="n">
+        <v>17</v>
+      </c>
+      <c r="E12" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="F12" s="5" t="n">
         <v>19</v>
       </c>
-      <c r="E12" s="5" t="n">
-        <v>16</v>
-      </c>
-      <c r="F12" s="5" t="n">
-        <v>21</v>
-      </c>
       <c r="G12" s="5" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="I12" s="6">
         <f>SUM(B12:H12)</f>
@@ -1957,10 +1957,10 @@
         <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E4" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5">
@@ -2020,10 +2020,10 @@
         <v>0</v>
       </c>
       <c r="D7" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E7" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8">
@@ -2062,10 +2062,10 @@
         <v>0</v>
       </c>
       <c r="D9" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E9" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="10">
@@ -2104,10 +2104,10 @@
         <v>0</v>
       </c>
       <c r="D11" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E11" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="12">
@@ -2125,10 +2125,10 @@
         <v>0</v>
       </c>
       <c r="D12" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E12" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="13">
@@ -2146,10 +2146,10 @@
         <v>0</v>
       </c>
       <c r="D13" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="E13" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="14">
@@ -2167,10 +2167,10 @@
         <v>0</v>
       </c>
       <c r="D14" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="E14" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="15">
@@ -2188,10 +2188,10 @@
         <v>8</v>
       </c>
       <c r="D15" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="E15" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="16">
@@ -2356,10 +2356,10 @@
         <v>10</v>
       </c>
       <c r="D23" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E23" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="24">
@@ -2377,10 +2377,10 @@
         <v>10</v>
       </c>
       <c r="D24" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E24" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="25">
@@ -2398,10 +2398,10 @@
         <v>16</v>
       </c>
       <c r="D25" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="E25" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="26">
@@ -2419,10 +2419,10 @@
         <v>16</v>
       </c>
       <c r="D26" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E26" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="27">
@@ -2440,10 +2440,10 @@
         <v>16</v>
       </c>
       <c r="D27" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="E27" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="28">
@@ -2461,10 +2461,10 @@
         <v>20</v>
       </c>
       <c r="D28" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="E28" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="29">
@@ -2482,10 +2482,10 @@
         <v>20</v>
       </c>
       <c r="D29" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="E29" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
KIDS: recorte final −15% por talla (×0.85)
Co-authored-by: scm-svg <scm-svg@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/PROPUESTA_PRODUCCION_SUBLIMADO_ACTUALIZADA.xlsx
+++ b/PROPUESTA_PRODUCCION_SUBLIMADO_ACTUALIZADA.xlsx
@@ -540,19 +540,19 @@
         <v>136</v>
       </c>
       <c r="C3" t="n">
-        <v>273</v>
+        <v>252</v>
       </c>
       <c r="D3" t="n">
-        <v>330</v>
+        <v>305</v>
       </c>
       <c r="E3" t="n">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="F3" t="n">
-        <v>20.9</v>
+        <v>21</v>
       </c>
       <c r="G3" t="n">
-        <v>137</v>
+        <v>116</v>
       </c>
     </row>
     <row r="4">
@@ -565,19 +565,19 @@
         <v>485</v>
       </c>
       <c r="C4" t="n">
-        <v>728</v>
+        <v>707</v>
       </c>
       <c r="D4" t="n">
-        <v>876</v>
+        <v>851</v>
       </c>
       <c r="E4" t="n">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="F4" t="n">
-        <v>20.3</v>
+        <v>20.4</v>
       </c>
       <c r="G4" t="n">
-        <v>243</v>
+        <v>222</v>
       </c>
     </row>
   </sheetData>
@@ -1043,10 +1043,10 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C6" s="5" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D6" s="5" t="n">
         <v>8</v>
@@ -1055,13 +1055,13 @@
         <v>4</v>
       </c>
       <c r="F6" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="G6" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="H6" s="5" t="n">
         <v>5</v>
-      </c>
-      <c r="G6" s="5" t="n">
-        <v>9</v>
-      </c>
-      <c r="H6" s="5" t="n">
-        <v>6</v>
       </c>
       <c r="I6" s="6">
         <f>SUM(B6:H6)</f>
@@ -1120,19 +1120,19 @@
         <v>4</v>
       </c>
       <c r="D8" s="5" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F8" s="5" t="n">
+        <v>16</v>
+      </c>
+      <c r="G8" s="5" t="n">
+        <v>18</v>
+      </c>
+      <c r="H8" s="5" t="n">
         <v>17</v>
-      </c>
-      <c r="G8" s="5" t="n">
-        <v>19</v>
-      </c>
-      <c r="H8" s="5" t="n">
-        <v>18</v>
       </c>
       <c r="I8" s="6">
         <f>SUM(B8:H8)</f>
@@ -1194,16 +1194,16 @@
         <v>4</v>
       </c>
       <c r="E10" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="F10" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="F10" s="5" t="n">
-        <v>6</v>
-      </c>
       <c r="G10" s="5" t="n">
         <v>4</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I10" s="6">
         <f>SUM(B10:H10)</f>
@@ -1256,25 +1256,25 @@
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C12" s="5" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D12" s="5" t="n">
+        <v>16</v>
+      </c>
+      <c r="E12" s="5" t="n">
+        <v>14</v>
+      </c>
+      <c r="F12" s="5" t="n">
+        <v>18</v>
+      </c>
+      <c r="G12" s="5" t="n">
+        <v>21</v>
+      </c>
+      <c r="H12" s="5" t="n">
         <v>17</v>
-      </c>
-      <c r="E12" s="5" t="n">
-        <v>15</v>
-      </c>
-      <c r="F12" s="5" t="n">
-        <v>19</v>
-      </c>
-      <c r="G12" s="5" t="n">
-        <v>23</v>
-      </c>
-      <c r="H12" s="5" t="n">
-        <v>18</v>
       </c>
       <c r="I12" s="6">
         <f>SUM(B12:H12)</f>
@@ -1915,10 +1915,10 @@
         <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3">
@@ -1936,10 +1936,10 @@
         <v>0</v>
       </c>
       <c r="D3" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E3" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4">
@@ -1999,10 +1999,10 @@
         <v>8</v>
       </c>
       <c r="D6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E6" t="n">
-        <v>-3</v>
+        <v>-4</v>
       </c>
     </row>
     <row r="7">
@@ -2020,10 +2020,10 @@
         <v>0</v>
       </c>
       <c r="D7" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E7" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="8">
@@ -2041,10 +2041,10 @@
         <v>0</v>
       </c>
       <c r="D8" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E8" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="9">
@@ -2104,10 +2104,10 @@
         <v>0</v>
       </c>
       <c r="D11" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E11" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="12">
@@ -2125,10 +2125,10 @@
         <v>0</v>
       </c>
       <c r="D12" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E12" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="13">
@@ -2146,10 +2146,10 @@
         <v>0</v>
       </c>
       <c r="D13" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E13" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="14">
@@ -2167,10 +2167,10 @@
         <v>0</v>
       </c>
       <c r="D14" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E14" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="15">
@@ -2188,10 +2188,10 @@
         <v>8</v>
       </c>
       <c r="D15" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E15" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="16">
@@ -2272,10 +2272,10 @@
         <v>0</v>
       </c>
       <c r="D19" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E19" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="20">
@@ -2293,10 +2293,10 @@
         <v>0</v>
       </c>
       <c r="D20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="21">
@@ -2335,10 +2335,10 @@
         <v>4</v>
       </c>
       <c r="D22" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E22" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23">
@@ -2356,10 +2356,10 @@
         <v>10</v>
       </c>
       <c r="D23" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E23" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="24">
@@ -2377,10 +2377,10 @@
         <v>10</v>
       </c>
       <c r="D24" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E24" t="n">
-        <v>-1</v>
+        <v>-2</v>
       </c>
     </row>
     <row r="25">
@@ -2398,10 +2398,10 @@
         <v>16</v>
       </c>
       <c r="D25" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E25" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26">
@@ -2419,10 +2419,10 @@
         <v>16</v>
       </c>
       <c r="D26" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E26" t="n">
-        <v>-1</v>
+        <v>-2</v>
       </c>
     </row>
     <row r="27">
@@ -2440,10 +2440,10 @@
         <v>16</v>
       </c>
       <c r="D27" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E27" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="28">
@@ -2461,10 +2461,10 @@
         <v>20</v>
       </c>
       <c r="D28" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="E28" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="29">
@@ -2482,10 +2482,10 @@
         <v>20</v>
       </c>
       <c r="D29" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E29" t="n">
-        <v>-2</v>
+        <v>-3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Alinear proporciones por talla al dashboard (periodo completo)
- Mix de ventas Oct–Sep (no solo meses velocidad): 14 y L lideran
- Rebalanceo final por color + ajuste L≥M (CAB) y 14≥12 (KIDS)
- Trim KIDS al final para no distorsionar curvas

Co-authored-by: scm-svg <scm-svg@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/PROPUESTA_PRODUCCION_SUBLIMADO_ACTUALIZADA.xlsx
+++ b/PROPUESTA_PRODUCCION_SUBLIMADO_ACTUALIZADA.xlsx
@@ -515,19 +515,19 @@
         <v>349</v>
       </c>
       <c r="C2" t="n">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="D2" t="n">
-        <v>546</v>
+        <v>544</v>
       </c>
       <c r="E2" t="n">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F2" t="n">
-        <v>20</v>
+        <v>19.8</v>
       </c>
       <c r="G2" t="n">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="3">
@@ -540,19 +540,19 @@
         <v>136</v>
       </c>
       <c r="C3" t="n">
-        <v>252</v>
+        <v>225</v>
       </c>
       <c r="D3" t="n">
-        <v>305</v>
+        <v>271</v>
       </c>
       <c r="E3" t="n">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="F3" t="n">
-        <v>21</v>
+        <v>20.4</v>
       </c>
       <c r="G3" t="n">
-        <v>116</v>
+        <v>89</v>
       </c>
     </row>
     <row r="4">
@@ -565,19 +565,19 @@
         <v>485</v>
       </c>
       <c r="C4" t="n">
-        <v>707</v>
+        <v>679</v>
       </c>
       <c r="D4" t="n">
-        <v>851</v>
+        <v>815</v>
       </c>
       <c r="E4" t="n">
-        <v>144</v>
+        <v>136</v>
       </c>
       <c r="F4" t="n">
-        <v>20.4</v>
+        <v>20</v>
       </c>
       <c r="G4" t="n">
-        <v>222</v>
+        <v>194</v>
       </c>
     </row>
   </sheetData>
@@ -664,19 +664,19 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C6" s="5" t="n">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="D6" s="5" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G6" s="6">
         <f>SUM(B6:F6)</f>
@@ -721,19 +721,19 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="C8" s="5" t="n">
+        <v>33</v>
+      </c>
+      <c r="D8" s="5" t="n">
+        <v>39</v>
+      </c>
+      <c r="E8" s="5" t="n">
+        <v>16</v>
+      </c>
+      <c r="F8" s="5" t="n">
         <v>12</v>
-      </c>
-      <c r="C8" s="5" t="n">
-        <v>34</v>
-      </c>
-      <c r="D8" s="5" t="n">
-        <v>38</v>
-      </c>
-      <c r="E8" s="5" t="n">
-        <v>14</v>
-      </c>
-      <c r="F8" s="5" t="n">
-        <v>15</v>
       </c>
       <c r="G8" s="6">
         <f>SUM(B8:F8)</f>
@@ -778,19 +778,19 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C10" s="5" t="n">
         <v>10</v>
       </c>
       <c r="D10" s="5" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="F10" s="5" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G10" s="6">
         <f>SUM(B10:F10)</f>
@@ -835,16 +835,16 @@
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C12" s="5" t="n">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="D12" s="5" t="n">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="F12" s="5" t="n">
         <v>25</v>
@@ -1043,25 +1043,25 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C6" s="5" t="n">
         <v>4</v>
       </c>
       <c r="D6" s="5" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E6" s="5" t="n">
         <v>4</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G6" s="5" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="I6" s="6">
         <f>SUM(B6:H6)</f>
@@ -1120,19 +1120,19 @@
         <v>4</v>
       </c>
       <c r="D8" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="E8" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="F8" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="G8" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="H8" s="5" t="n">
         <v>9</v>
-      </c>
-      <c r="E8" s="5" t="n">
-        <v>9</v>
-      </c>
-      <c r="F8" s="5" t="n">
-        <v>16</v>
-      </c>
-      <c r="G8" s="5" t="n">
-        <v>18</v>
-      </c>
-      <c r="H8" s="5" t="n">
-        <v>17</v>
       </c>
       <c r="I8" s="6">
         <f>SUM(B8:H8)</f>
@@ -1194,13 +1194,13 @@
         <v>4</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F10" s="5" t="n">
         <v>5</v>
       </c>
       <c r="G10" s="5" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H10" s="5" t="n">
         <v>5</v>
@@ -1256,25 +1256,25 @@
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C12" s="5" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D12" s="5" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="E12" s="5" t="n">
         <v>14</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="G12" s="5" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="I12" s="6">
         <f>SUM(B12:H12)</f>
@@ -1454,10 +1454,10 @@
         <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E2" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="3">
@@ -1475,10 +1475,10 @@
         <v>24</v>
       </c>
       <c r="D3" t="n">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="E3" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4">
@@ -1496,10 +1496,10 @@
         <v>28</v>
       </c>
       <c r="D4" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E4" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5">
@@ -1517,10 +1517,10 @@
         <v>10</v>
       </c>
       <c r="D5" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="E5" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6">
@@ -1538,10 +1538,10 @@
         <v>10</v>
       </c>
       <c r="D6" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7">
@@ -1559,10 +1559,10 @@
         <v>0</v>
       </c>
       <c r="D7" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E7" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="8">
@@ -1580,10 +1580,10 @@
         <v>15</v>
       </c>
       <c r="D8" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E8" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="9">
@@ -1601,10 +1601,10 @@
         <v>30</v>
       </c>
       <c r="D9" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E9" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="10">
@@ -1622,10 +1622,10 @@
         <v>21</v>
       </c>
       <c r="D10" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="E10" t="n">
-        <v>-7</v>
+        <v>-5</v>
       </c>
     </row>
     <row r="11">
@@ -1643,10 +1643,10 @@
         <v>16</v>
       </c>
       <c r="D11" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="E11" t="n">
-        <v>-1</v>
+        <v>-4</v>
       </c>
     </row>
     <row r="12">
@@ -1664,10 +1664,10 @@
         <v>0</v>
       </c>
       <c r="D12" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E12" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="13">
@@ -1706,10 +1706,10 @@
         <v>15</v>
       </c>
       <c r="D14" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E14" t="n">
-        <v>-5</v>
+        <v>-4</v>
       </c>
     </row>
     <row r="15">
@@ -1727,10 +1727,10 @@
         <v>0</v>
       </c>
       <c r="D15" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="E15" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
     </row>
     <row r="16">
@@ -1748,10 +1748,10 @@
         <v>0</v>
       </c>
       <c r="D16" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E16" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="17">
@@ -1769,10 +1769,10 @@
         <v>20</v>
       </c>
       <c r="D17" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18">
@@ -1790,10 +1790,10 @@
         <v>45</v>
       </c>
       <c r="D18" t="n">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="E18" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
     </row>
     <row r="19">
@@ -1811,10 +1811,10 @@
         <v>45</v>
       </c>
       <c r="D19" t="n">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E19" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="20">
@@ -1832,10 +1832,10 @@
         <v>35</v>
       </c>
       <c r="D20" t="n">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="E20" t="n">
-        <v>-3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21">
@@ -1915,10 +1915,10 @@
         <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3">
@@ -1957,10 +1957,10 @@
         <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="5">
@@ -1999,10 +1999,10 @@
         <v>8</v>
       </c>
       <c r="D6" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E6" t="n">
-        <v>-4</v>
+        <v>-2</v>
       </c>
     </row>
     <row r="7">
@@ -2020,10 +2020,10 @@
         <v>0</v>
       </c>
       <c r="D7" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E7" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8">
@@ -2041,10 +2041,10 @@
         <v>0</v>
       </c>
       <c r="D8" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="E8" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9">
@@ -2104,10 +2104,10 @@
         <v>0</v>
       </c>
       <c r="D11" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="E11" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
     </row>
     <row r="12">
@@ -2125,10 +2125,10 @@
         <v>0</v>
       </c>
       <c r="D12" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="E12" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="13">
@@ -2146,10 +2146,10 @@
         <v>0</v>
       </c>
       <c r="D13" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="E13" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
     </row>
     <row r="14">
@@ -2167,10 +2167,10 @@
         <v>0</v>
       </c>
       <c r="D14" t="n">
-        <v>18</v>
+        <v>7</v>
       </c>
       <c r="E14" t="n">
-        <v>18</v>
+        <v>7</v>
       </c>
     </row>
     <row r="15">
@@ -2188,10 +2188,10 @@
         <v>8</v>
       </c>
       <c r="D15" t="n">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="E15" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16">
@@ -2272,10 +2272,10 @@
         <v>0</v>
       </c>
       <c r="D19" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E19" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="20">
@@ -2314,10 +2314,10 @@
         <v>0</v>
       </c>
       <c r="D21" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E21" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="22">
@@ -2356,10 +2356,10 @@
         <v>10</v>
       </c>
       <c r="D23" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="E23" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="24">
@@ -2377,10 +2377,10 @@
         <v>10</v>
       </c>
       <c r="D24" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E24" t="n">
-        <v>-2</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="25">
@@ -2398,10 +2398,10 @@
         <v>16</v>
       </c>
       <c r="D25" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="E25" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
     </row>
     <row r="26">
@@ -2440,10 +2440,10 @@
         <v>16</v>
       </c>
       <c r="D27" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E27" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28">
@@ -2461,10 +2461,10 @@
         <v>20</v>
       </c>
       <c r="D28" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="E28" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="29">
@@ -2482,10 +2482,10 @@
         <v>20</v>
       </c>
       <c r="D29" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="E29" t="n">
-        <v>-3</v>
+        <v>-1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>